<commit_message>
Add consumer data capture and marketing messaging to the chess challenge
- scripts/game-events.js: PII-free game events pushed to
  window.adobeDataLayer and, for registered players, to POST /events.
- Registration sends a consent context (page, experiment, variant); the
  session keeps only the marketing opt-in flag.
- player-message block: on-site marketing message for the current visit,
  one authored item per audience (registered, waiting, won, lost, draw),
  opted-in players only, {firstName} from game data, unsubscribe notice.
- Copy: new placeholders and post-game follow-up email copy (3 locales,
  fr/fr machine translated), message items on all six pages.
- Contract v1.1 (events, consent record, connectors, follow-up email,
  unsubscribe) and docs/backend-marketing-prompt.md for App Builder.
- Architecture diagrams and README updated.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-chess-challenge.report.xlsx
+++ b/tools/importer/reports/import-chess-challenge.report.xlsx
@@ -127,7 +127,7 @@
     <t>fr/fr/chess-challenge.report.json</t>
   </si>
   <si>
-    <t>["age-gate","player-registration","chess","invite"]</t>
+    <t>["age-gate","player-registration","chess","invite","player-message"]</t>
   </si>
   <si>
     <t>fr/fr/chess-challenge</t>
@@ -136,7 +136,7 @@
     <t>chess-challenge</t>
   </si>
   <si>
-    <t>2026-10-16T13:36:39.459Z</t>
+    <t>2026-10-21T09:30:31.524Z</t>
   </si>
   <si>
     <t>Le Suze Chess Challenge</t>
@@ -154,7 +154,7 @@
     <t>masters/en/chess-challenge</t>
   </si>
   <si>
-    <t>2026-10-16T13:36:29.433Z</t>
+    <t>2026-10-21T09:30:21.631Z</t>
   </si>
   <si>
     <t>The Suze Chess Challenge</t>
@@ -169,7 +169,7 @@
     <t>us/es/chess-challenge</t>
   </si>
   <si>
-    <t>2026-10-16T13:36:33.656Z</t>
+    <t>2026-10-21T09:30:25.922Z</t>
   </si>
   <si>
     <t>El Suze Chess Challenge</t>
@@ -184,7 +184,7 @@
     <t>experiments/fr/fr/chess-challenge/exp-chess-001/challenger</t>
   </si>
   <si>
-    <t>2026-10-16T13:36:53.830Z</t>
+    <t>2026-10-21T09:30:44.469Z</t>
   </si>
   <si>
     <t>http://localhost:3000/tools/importer/sources/chess-challenge/fr-fr.html?variant=challenger</t>
@@ -199,7 +199,7 @@
     <t>experiments/masters/en/chess-challenge/exp-chess-001/challenger</t>
   </si>
   <si>
-    <t>2026-10-16T13:36:44.487Z</t>
+    <t>2026-10-21T09:30:35.169Z</t>
   </si>
   <si>
     <t>http://localhost:3000/tools/importer/sources/chess-challenge/masters-en.html?variant=challenger</t>
@@ -211,7 +211,7 @@
     <t>experiments/us/es/chess-challenge/exp-chess-001/challenger</t>
   </si>
   <si>
-    <t>2026-10-16T13:36:48.610Z</t>
+    <t>2026-10-21T09:30:40.224Z</t>
   </si>
   <si>
     <t>http://localhost:3000/tools/importer/sources/chess-challenge/us-es.html?variant=challenger</t>

</xml_diff>

<commit_message>
Make us/en the English game market; masters/en is the unpublished blueprint
- Game locales are us/en, us/es and fr/fr. masters/en/chess-challenge is the
  MSM blueprint (no experiment, conversion setting inherited) rolled out to
  us/en, where the experiment is set locally.
- Import: new us-en source generating only the us/en challenger
  (/experiments/us/en/..., date-of-birth age gate 21, nudge); the masters
  challenger is no longer generated; experiment metadata only when defined.
- tools/importer/clean-jcr-export.mjs (npm run export:clean): keeps only
  the chess pages in the AEM export. Every import regenerates July leftovers
  (empty masters/fr parents, France/English snapshots) that wiped the
  blueprints and broke MSM live copies when pushed.
- Default locale fallback, contract and backend prompts now use us/en.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-chess-challenge.report.xlsx
+++ b/tools/importer/reports/import-chess-challenge.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="72">
   <si>
     <t>_reportFile</t>
   </si>
@@ -136,7 +136,7 @@
     <t>chess-challenge</t>
   </si>
   <si>
-    <t>2026-10-21T09:30:31.524Z</t>
+    <t>2026-10-26T09:32:36.990Z</t>
   </si>
   <si>
     <t>Le Suze Chess Challenge</t>
@@ -154,7 +154,7 @@
     <t>masters/en/chess-challenge</t>
   </si>
   <si>
-    <t>2026-10-21T09:30:21.631Z</t>
+    <t>2026-10-26T09:32:28.854Z</t>
   </si>
   <si>
     <t>The Suze Chess Challenge</t>
@@ -169,7 +169,7 @@
     <t>us/es/chess-challenge</t>
   </si>
   <si>
-    <t>2026-10-21T09:30:25.922Z</t>
+    <t>2026-10-26T09:32:32.985Z</t>
   </si>
   <si>
     <t>El Suze Chess Challenge</t>
@@ -184,7 +184,7 @@
     <t>experiments/fr/fr/chess-challenge/exp-chess-001/challenger</t>
   </si>
   <si>
-    <t>2026-10-21T09:30:44.469Z</t>
+    <t>2026-10-26T09:32:48.300Z</t>
   </si>
   <si>
     <t>http://localhost:3000/tools/importer/sources/chess-challenge/fr-fr.html?variant=challenger</t>
@@ -205,13 +205,25 @@
     <t>http://localhost:3000/tools/importer/sources/chess-challenge/masters-en.html?variant=challenger</t>
   </si>
   <si>
+    <t>experiments/us/en/chess-challenge/exp-chess-001/challenger.report.json</t>
+  </si>
+  <si>
+    <t>experiments/us/en/chess-challenge/exp-chess-001/challenger</t>
+  </si>
+  <si>
+    <t>2026-10-26T09:32:52.621Z</t>
+  </si>
+  <si>
+    <t>http://localhost:3000/tools/importer/sources/chess-challenge/us-en.html?variant=challenger</t>
+  </si>
+  <si>
     <t>experiments/us/es/chess-challenge/exp-chess-001/challenger.report.json</t>
   </si>
   <si>
     <t>experiments/us/es/chess-challenge/exp-chess-001/challenger</t>
   </si>
   <si>
-    <t>2026-10-21T09:30:40.224Z</t>
+    <t>2026-10-26T09:32:42.479Z</t>
   </si>
   <si>
     <t>http://localhost:3000/tools/importer/sources/chess-challenge/us-es.html?variant=challenger</t>
@@ -603,7 +615,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -923,12 +935,41 @@
         <v>66</v>
       </c>
       <c r="G11" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="H11" t="s">
         <v>67</v>
       </c>
       <c r="I11" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" t="s">
+        <v>69</v>
+      </c>
+      <c r="D12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" t="s">
+        <v>40</v>
+      </c>
+      <c r="F12" t="s">
+        <v>70</v>
+      </c>
+      <c r="G12" t="s">
+        <v>53</v>
+      </c>
+      <c r="H12" t="s">
+        <v>71</v>
+      </c>
+      <c r="I12" t="s">
         <v>59</v>
       </c>
     </row>

</xml_diff>